<commit_message>
Corrected Case on folders
</commit_message>
<xml_diff>
--- a/Assets/Data/Amstrad CPC 664/MC0005A/Data CPC 664 MC0005A v2.0.0.xlsx
+++ b/Assets/Data/Amstrad CPC 664/MC0005A/Data CPC 664 MC0005A v2.0.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbewe\AppData\Local\Classic-Repair-Toolbox\Data\Amstrad CPC 664\MC0005A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACE534C-8BF0-4E96-9919-7D2BAA828587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFEAD5D-45B7-436E-895E-3B4E9DD099CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EBC5E150-CC27-441B-9E4F-9F7CF77570D6}"/>
   </bookViews>
@@ -1907,262 +1907,262 @@
     <t>Thumbnail highlight color</t>
   </si>
   <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC107_14_PC0.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC108_4_MA0.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC108_18_DISPEN.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC108_38_RA0.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC108_39_HSYNC.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC108_40_VSYNC.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_1_A11.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_2_A12.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_3_A13.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_4_A14.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_5_A15.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_6_CLK.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_7_D4.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_8_D3.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_9_D5.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_10_D6.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_12_D2.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_13_D7.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_14_D0.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_15_D1.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_16_INT.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_17_NMI.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_18_HALT.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_19_MREQ.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_20_IORQ.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_21_RD.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_22_WR.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_23_BUSAK.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_24_WAIT.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_25_BUSRQ.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_26_RESET.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_27_M1.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_28_RFSH.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_30_A0.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_31_A1.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_32_A2.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_33_A3.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_34_A4.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_35_A5.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_36_A6.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_37_A7.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_38_A8.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_39_A9.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC111_40_A10.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_4_CCLK.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_5_NSYNC.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_8_B.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_10_G.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_12_R.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_14_NCPU.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_16_NCAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_19_NPHI.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_23_N244EN.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_24_CK16.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_31_NCASAD.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_33_NMWE.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC116_34_NRAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC117_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC117_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC117_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC118_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC118_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC118_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC119_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC119_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC119_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC120_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC120_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC120_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC121_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC121_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC121_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC122_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC122_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC122_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC123_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC123_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC123_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC124_3_W.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC124_4_RAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/IC124_15_CAS.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Scope Baseline/X101_1_CLK.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Truth Tables/IC104_TRUTH_TABLE.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Truth Tables/IC105_TRUTH_TABLE.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Truth Tables/IC109_TRUTH_TABLE.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad CPC 664/MC0005A/Truth Tables/IC113_TRUTH_TABLE.jpg</t>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC107_14_PC0.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC108_4_MA0.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC108_18_DISPEN.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC108_38_RA0.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC108_39_HSYNC.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC108_40_VSYNC.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_1_A11.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_2_A12.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_3_A13.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_4_A14.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_5_A15.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_6_CLK.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_7_D4.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_8_D3.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_9_D5.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_10_D6.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_12_D2.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_13_D7.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_14_D0.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_15_D1.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_16_INT.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_17_NMI.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_18_HALT.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_19_MREQ.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_20_IORQ.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_21_RD.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_22_WR.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_23_BUSAK.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_24_WAIT.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_25_BUSRQ.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_26_RESET.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_27_M1.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_28_RFSH.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_30_A0.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_31_A1.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_32_A2.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_33_A3.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_34_A4.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_35_A5.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_36_A6.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_37_A7.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_38_A8.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_39_A9.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC111_40_A10.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_4_CCLK.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_5_NSYNC.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_8_B.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_10_G.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_12_R.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_14_NCPU.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_16_NCAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_19_NPHI.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_23_N244EN.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_24_CK16.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_31_NCASAD.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_33_NMWE.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC116_34_NRAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC117_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC117_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC117_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC118_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC118_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC118_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC119_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC119_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC119_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC120_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC120_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC120_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC121_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC121_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC121_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC122_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC122_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC122_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC123_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC123_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC123_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC124_3_W.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC124_4_RAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/IC124_15_CAS.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Scope baseline/X101_1_CLK.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Truth tables/IC104_TRUTH_TABLE.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Truth tables/IC105_TRUTH_TABLE.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Truth tables/IC109_TRUTH_TABLE.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad CPC 664/MC0005A/Truth tables/IC113_TRUTH_TABLE.jpg</t>
   </si>
   <si>
     <r>
@@ -2177,7 +2177,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>2026-May-7</t>
+      <t>2026-May-8</t>
     </r>
   </si>
 </sst>

</xml_diff>